<commit_message>
sims: LP-economics v2 — formatter polish + auditor fixes applied
Formatter (sonnet): banners, freeze panes, widths, number formats, legends,
green/red legend, one LineChart; manager-verified ALL 156 cells' formulas +
9 assumption values byte-identical pre/post (0 changed), chart intact.

Auditor (skeptic, opus): arithmetic clean; fixes applied on top —
- protection_factor DEFAULT 0.5 -> 0 (kills the protection/funding
  double-count; conservative headline);
- funding_APR note: can be NEGATIVE (LP paying side);
- break-even note clarified (levered-zero, opportunity cost);
- READ_ME AUDITED caveat.
Conservative grid honestly shows LPs wiped (-27%) in high-vol/low-turnover.
NON-CORE (sims/). NOTES updated with the audit table.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cs1cJ4yQMcmxqbEVrDpqHd
</commit_message>
<xml_diff>
--- a/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
+++ b/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
@@ -19,11 +19,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot; bps&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0&quot;×&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +50,73 @@
       <color rgb="00555555"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="002B6CB0"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A365D"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002D3748"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A202C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A202C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002B6CB0"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A365D"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -76,8 +143,18 @@
         <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -99,11 +176,39 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D69E2E"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D69E2E"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D69E2E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D69E2E"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,6 +223,81 @@
     <xf numFmtId="165" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -208,6 +388,280 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>BASE net APR vs daily turnover (by sigma)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Regime_Grid'!$A$3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Regime_Grid'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Regime_Grid'!$B$3:$F$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Regime_Grid'!$A$4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Regime_Grid'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Regime_Grid'!$B$4:$F$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Regime_Grid'!$A$5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Regime_Grid'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Regime_Grid'!$B$5:$F$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Regime_Grid'!$A$6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Regime_Grid'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Regime_Grid'!$B$6:$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Regime_Grid'!$A$7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Regime_Grid'!$B$2:$F$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Regime_Grid'!$B$7:$F$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>daily turnover</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>net APR</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -502,21 +956,25 @@
   <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="115" customWidth="1" min="1" max="1"/>
+    <col width="118" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Temporal LP economics — editable model (v2, +LP leverage) — BRAINSTORM / non-core</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>AUDITED (opus): arithmetic clean. Defaults set CONSERVATIVE (protection_factor=0) so the green grid is NOT an optimism-on headline. funding_APR &amp; protection_factor are UNPROVEN placeholders and can double-count — keep them separate.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Edit the YELLOW cells on 'Assumptions'. Everything recomputes. Open in Excel / Google Sheets / LibreOffice.</t>
         </is>
@@ -526,42 +984,42 @@
       <c r="A4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>MODEL (per $ of equity, annualized):</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  Temporal_net = fee_bps/10000·turnover·days + funding_APR − (sigma^2/8)·(1−protection) − drain·turnover</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  Levered_Temporal = LP_leverage·Temporal_net − (LP_leverage−1)·borrow_APR   [leverage acts ONLY on the Temporal part]</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  HLP_layer = HLP_base_APR·(1 − HLP_tail_haircut·sigma)   [additive, at MARGIN level, NOT levered]</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  BASE (dollar margin)   net APR = Levered_Temporal</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  RESTAKED (HLP margin)  net APR = Levered_Temporal + HLP_layer</t>
         </is>
@@ -571,48 +1029,51 @@
       <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>HONESTY LABELS:</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  - funding_APR = STAND-IN for the update-2 funding formula (undecided). protection_factor = unproven hypothesis.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Leverage cuts BOTH ways: if Temporal_net &lt; borrow_APR, leverage makes it WORSE. And it raises liquidation risk</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">    in high vol (a levered LVR loss &gt; 1/leverage of equity wipes you) — the sheet does NOT model liquidation; caveat only.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  - HLP is NOT levered (operator: additive at margin). HLP_tail_haircut&gt;0 models HLP+Temporal losing together in crashes.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Reduced-form sketch, NOT a validated backtest. Lives in sims/ (non-core).</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -623,225 +1084,241 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>EDITABLE ASSUMPTIONS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>Disclosure / note</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>days_per_year</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="21" t="n">
         <v>365</v>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>trading days/year</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>fee_bps</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>taker fee, bps of notional traded. 0 if no fee (TBD).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>funding_APR</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="26" t="n">
         <v>0.03</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>NET funding income/yr to LP (PLACEHOLDER for update-2 formula). Main edge vs vanilla AMM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>NET funding income/yr to LP (PLACEHOLDER for update-2 formula). CAN BE NEGATIVE when the LP is on the paying side of funding. The hypothesized edge vs a vanilla AMM — unproven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>protection_factor</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>WARP-only LVR reduction (0..1). DEFAULT 0 = no assumed reduction (conservative). Do NOT also attribute the funding tether here — that is funding_APR; counting both DOUBLE-COUNTS. Unproven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>drain_coeff</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>round-trip drain APR per 1.0 daily turnover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>HLP_base_APR</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>yield on HLP margin (external). NOT levered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>HLP_tail_haircut</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>0=pure additive; &gt;0 shaves HLP yield as vol rises (crash co-movement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>LP_leverage</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>leverage on the TEMPORAL position (equity ×L exposure). Does NOT apply to HLP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>borrow_APR</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>cost of the borrowed (L−1) leg, e.g. stablecoin borrow rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Grid axes (editable):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>daily_turnover -&gt;</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C15" s="27" t="n">
         <v>0.5</v>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>fraction of LVR removed by warp+funding tether. 0..1. HYPOTHESIS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>drain_coeff</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>round-trip drain APR per 1.0 daily turnover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>HLP_base_APR</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>yield on HLP margin (external). NOT levered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>HLP_tail_haircut</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>0=pure additive; &gt;0 shaves HLP yield as vol rises (crash co-movement).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>LP_leverage</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
+      <c r="D15" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>leverage on the TEMPORAL position (equity ×L exposure). Does NOT apply to HLP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>borrow_APR</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>cost of the borrowed (L−1) leg, e.g. stablecoin borrow rate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Grid axes (editable):</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>daily_turnover -&gt;</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" s="9" t="n">
+      <c r="F15" s="27" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>sigma (annualized) -&gt;</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="26" t="n">
         <v>0.4</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="26" t="n">
         <v>0.9</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="26" t="n">
         <v>1.2</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>LEGEND:</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>yellow fill = editable input cell</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A14:C14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -852,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -863,342 +1340,359 @@
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>LEVERED LP (dollar margin) — net yield APR. GREEN=profit, RED=loss.</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>sigma \ turnover(/day)</t>
         </is>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="34">
         <f>Assumptions!B$15</f>
         <v/>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="34">
         <f>Assumptions!C$15</f>
         <v/>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="34">
         <f>Assumptions!D$15</f>
         <v/>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="34">
         <f>Assumptions!E$15</f>
         <v/>
       </c>
-      <c r="F2" s="10">
+      <c r="F2" s="34">
         <f>Assumptions!F$15</f>
         <v/>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="11">
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="35">
         <f>Assumptions!B$16</f>
         <v/>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$2*Assumptions!$B$4+Assumptions!$B$6-(($A3^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$2*Assumptions!$B$4+Assumptions!$B$6-(($A3^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$2*Assumptions!$B$4+Assumptions!$B$6-(($A3^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$2*Assumptions!$B$4+Assumptions!$B$6-(($A3^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$2*Assumptions!$B$4+Assumptions!$B$6-(($A3^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="11">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="35">
         <f>Assumptions!C$16</f>
         <v/>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$2*Assumptions!$B$4+Assumptions!$B$6-(($A4^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$2*Assumptions!$B$4+Assumptions!$B$6-(($A4^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$2*Assumptions!$B$4+Assumptions!$B$6-(($A4^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$2*Assumptions!$B$4+Assumptions!$B$6-(($A4^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$2*Assumptions!$B$4+Assumptions!$B$6-(($A4^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11">
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="35">
         <f>Assumptions!D$16</f>
         <v/>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$2*Assumptions!$B$4+Assumptions!$B$6-(($A5^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$2*Assumptions!$B$4+Assumptions!$B$6-(($A5^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$2*Assumptions!$B$4+Assumptions!$B$6-(($A5^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$2*Assumptions!$B$4+Assumptions!$B$6-(($A5^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$2*Assumptions!$B$4+Assumptions!$B$6-(($A5^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="11">
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="35">
         <f>Assumptions!E$16</f>
         <v/>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$2*Assumptions!$B$4+Assumptions!$B$6-(($A6^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$2*Assumptions!$B$4+Assumptions!$B$6-(($A6^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$2*Assumptions!$B$4+Assumptions!$B$6-(($A6^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$2*Assumptions!$B$4+Assumptions!$B$6-(($A6^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$2*Assumptions!$B$4+Assumptions!$B$6-(($A6^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="11">
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="35">
         <f>Assumptions!F$16</f>
         <v/>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$2*Assumptions!$B$4+Assumptions!$B$6-(($A7^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$2*Assumptions!$B$4+Assumptions!$B$6-(($A7^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$2*Assumptions!$B$4+Assumptions!$B$6-(($A7^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$2*Assumptions!$B$4+Assumptions!$B$6-(($A7^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$2*Assumptions!$B$4+Assumptions!$B$6-(($A7^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$2)-(Assumptions!$B$11-1)*Assumptions!$B$12)</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>LEVERED + RESTAKED (HLP margin) — net yield APR.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>sigma \ turnover(/day)</t>
         </is>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="34">
         <f>Assumptions!B$15</f>
         <v/>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="34">
         <f>Assumptions!C$15</f>
         <v/>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="34">
         <f>Assumptions!D$15</f>
         <v/>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="34">
         <f>Assumptions!E$15</f>
         <v/>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="34">
         <f>Assumptions!F$15</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="11">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="35">
         <f>Assumptions!B$16</f>
         <v/>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$11*Assumptions!$B$4+Assumptions!$B$6-(($A12^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A12)</f>
         <v/>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$11*Assumptions!$B$4+Assumptions!$B$6-(($A12^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A12)</f>
         <v/>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$11*Assumptions!$B$4+Assumptions!$B$6-(($A12^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A12)</f>
         <v/>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$11*Assumptions!$B$4+Assumptions!$B$6-(($A12^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A12)</f>
         <v/>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$11*Assumptions!$B$4+Assumptions!$B$6-(($A12^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A12)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="35">
         <f>Assumptions!C$16</f>
         <v/>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$11*Assumptions!$B$4+Assumptions!$B$6-(($A13^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A13)</f>
         <v/>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$11*Assumptions!$B$4+Assumptions!$B$6-(($A13^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A13)</f>
         <v/>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$11*Assumptions!$B$4+Assumptions!$B$6-(($A13^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A13)</f>
         <v/>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$11*Assumptions!$B$4+Assumptions!$B$6-(($A13^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A13)</f>
         <v/>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$11*Assumptions!$B$4+Assumptions!$B$6-(($A13^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A13)</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="11">
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="35">
         <f>Assumptions!D$16</f>
         <v/>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$11*Assumptions!$B$4+Assumptions!$B$6-(($A14^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A14)</f>
         <v/>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$11*Assumptions!$B$4+Assumptions!$B$6-(($A14^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A14)</f>
         <v/>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$11*Assumptions!$B$4+Assumptions!$B$6-(($A14^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A14)</f>
         <v/>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$11*Assumptions!$B$4+Assumptions!$B$6-(($A14^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A14)</f>
         <v/>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$11*Assumptions!$B$4+Assumptions!$B$6-(($A14^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A14)</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="35">
         <f>Assumptions!E$16</f>
         <v/>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$11*Assumptions!$B$4+Assumptions!$B$6-(($A15^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A15)</f>
         <v/>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$11*Assumptions!$B$4+Assumptions!$B$6-(($A15^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A15)</f>
         <v/>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$11*Assumptions!$B$4+Assumptions!$B$6-(($A15^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A15)</f>
         <v/>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$11*Assumptions!$B$4+Assumptions!$B$6-(($A15^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A15)</f>
         <v/>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$11*Assumptions!$B$4+Assumptions!$B$6-(($A15^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A15)</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="35">
         <f>Assumptions!F$16</f>
         <v/>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*B$11*Assumptions!$B$4+Assumptions!$B$6-(($A16^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*B$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A16)</f>
         <v/>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*C$11*Assumptions!$B$4+Assumptions!$B$6-(($A16^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*C$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A16)</f>
         <v/>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*D$11*Assumptions!$B$4+Assumptions!$B$6-(($A16^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*D$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A16)</f>
         <v/>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*E$11*Assumptions!$B$4+Assumptions!$B$6-(($A16^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*E$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A16)</f>
         <v/>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="36">
         <f>(Assumptions!$B$11*(Assumptions!$B$5/10000*F$11*Assumptions!$B$4+Assumptions!$B$6-(($A16^2)/8)*(1-Assumptions!$B$7)-Assumptions!$B$8*F$11)-(Assumptions!$B$11-1)*Assumptions!$B$12)+Assumptions!$B$9*(1-Assumptions!$B$10*$A16)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Break-even = green/red boundary. NB leverage helps only where Temporal_net &gt; borrow_APR; else it worsens losses.</t>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>Break-even = green/red boundary = LEVERED break-even (Temporal_net vs borrow_APR), not zero-Temporal; ignores opportunity cost. Defaults are CONSERVATIVE (protection=0); raise protection/funding to see the hypothesis-on case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>LEGEND:</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>green = LP profits (net APR &gt; 0)     red = LP loses (net APR &lt; 0)     inputs are edited on the Assumptions sheet</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A10:F10"/>
+  </mergeCells>
   <conditionalFormatting sqref="B3:F7">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -1216,6 +1710,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1225,141 +1720,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="58" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>SINGLE-SCENARIO BREAKDOWN (edit the two yellow inputs)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>daily_turnover</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="27" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>sigma (annualized)</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="26" t="n">
         <v>0.6</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>Fee income</t>
         </is>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="36">
         <f>Assumptions!$B$5/10000*$B$3*Assumptions!$B$4</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Funding income</t>
         </is>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="40">
         <f>Assumptions!$B$6</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="38" t="inlineStr">
         <is>
           <t>LVR cost</t>
         </is>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="36">
         <f>-(($B$4^2)/8)*(1-Assumptions!$B$7)</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="39" t="inlineStr">
         <is>
           <t>Round-trip drain</t>
         </is>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="40">
         <f>-Assumptions!$B$8*$B$3</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="38" t="inlineStr">
         <is>
           <t>Temporal_net (unlevered)</t>
         </is>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="36">
         <f>B6+B7+B8+B9</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="39" t="inlineStr">
         <is>
           <t>Levered Temporal</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="40">
         <f>Assumptions!$B$11*B10-(Assumptions!$B$11-1)*Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>HLP layer (unlevered, margin)</t>
         </is>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="36">
         <f>Assumptions!$B$9*(1-Assumptions!$B$10*$B$4)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="41" t="inlineStr">
         <is>
           <t>BASE levered net (dollar margin)</t>
         </is>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="42">
         <f>B11</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>RESTAKED levered net (HLP margin)</t>
         </is>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="42">
         <f>B11+B12</f>
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>LEGEND:</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>yellow fill = editable input cell</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
sims: add simplifying-assumptions / further-work disclaimer (entry 488)
Operator keeps hedge_funding_APR neutral (0) for simplicity; asks for
disclaimers. Added a "SIMPLIFYING ASSUMPTIONS — to be addressed in further
work" block to the xlsx READ_ME + NOTES (hedge funding neutral, clean/fee-
neutral hedge, funding placeholder, protection=0, LVR baseline, no
liquidation, HLP additive, reduced-form). Doc-only; formulas + chart
verified unchanged. NON-CORE. Transcript 488.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cs1cJ4yQMcmxqbEVrDpqHd
</commit_message>
<xml_diff>
--- a/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
+++ b/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
@@ -800,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -938,6 +938,83 @@
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  Reduced-form sketch, NOT a backtest. Lives in sims/ (non-core).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>SIMPLIFYING ASSUMPTIONS (v2.1) — to be addressed in FURTHER WORK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>1. Hedge-leg funding assumed NEUTRAL (hedge_funding_APR = 0). Real Hyperliquid hedge funding can be + or - and is not modeled here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>2. Delta hedge assumed clean &amp; fee-neutral: no tracking error, no discrete-rebalance slippage; hedge_fee_cost = 0 (maker approx taker).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>3. funding_APR is a PLACEHOLDER for the (undecided) update-2 funding formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>4. protection_factor = 0 (no assumed warp LVR-reduction); unproven if raised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>5. LVR = sigma^2/8 is the 50/50 CPMM baseline; Temporal is warped, so this is an approximation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>6. Liquidation of the levered leg is not modeled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>7. HLP treated as additive; tail-correlation off at default (HLP_tail_haircut = 0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>8. Reduced-form, annualized sketch — NOT a path-dependent backtest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Further work: plug realistic HL hedge-leg funding; model tracking error &amp; discrete rebalancing; derive funding_APR from the</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>update-2 formula; validate protection_factor; add liquidation + HLP tail-correlation; Monte-Carlo paths.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sims: FAITHFULNESS GAP — sim is a spot-AMM proxy, not the options AMM (entry 490)
Operator caught it: Temporal is a perp-OPTIONS AMM, not spot Balancer, so the
generic fees+funding−(σ²/8 LVR) model is NOT faithful. Recorded the gap in
xlsx READ_ME + NOTES: faithful model = LP as option SELLER — premium(IV) −
gamma bleed(RV, coefficient from the actual γ/m curve + open notional) +
funding/fees − hedge. Corrected the earlier "m is a read lens, vol cost
unchanged" claim (m DOES drive vol cost via the book's gamma). Chart/formulas
verified unchanged. Faithful rebuild pending operator go. Transcript 490.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cs1cJ4yQMcmxqbEVrDpqHd
</commit_message>
<xml_diff>
--- a/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
+++ b/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,11 @@
       <i val="1"/>
       <color rgb="00555555"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C53030"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="7">
@@ -129,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -171,6 +176,7 @@
     <xf numFmtId="165" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -800,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -941,6 +947,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
@@ -1015,6 +1022,55 @@
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>update-2 formula; validate protection_factor; add liquidation + HLP tail-correlation; Monte-Carlo paths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>FAITHFULNESS CAVEAT (operator entry 490) — READ THIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>This is a GENERIC spot-AMM-LP model (fees + funding − LVR), NOT a faithful perp-OPTIONS-AMM model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>A faithful version treats the LP as an option SELLER: revenue = option PREMIUM (at implied vol) + funding + fees;</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>volatility cost = the GAMMA bleed of the option book (coefficient set by the curve shape gamma &amp; m and open</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>notional), NOT the plain-pool sigma^2/8. In that faithful view the curve-shape knob m DOES drive the vol cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>The sigma^2 scaling is right; the 1/8 coefficient, the premium income, and the gamma/m dependence are the gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Rebuild pending operator go. Until then, read this sheet as a rough proxy, not the actual thing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sims+transcript: faithfulness gap is orthogonal to shape/steepness (entry 491)
Operator: the faithfulness question was orthogonal to the m/shape thing.
Restated cleanly in xlsx READ_ME + NOTES: sim is unfaithful because it is a
SPOT-AMM proxy, not an OPTIONS-AMM (LP sells options → premium income +
short-gamma vol cost + hedge), independent of the curve shape; dropped the m
tangent. Chart/formulas verified unchanged. Transcript 491.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cs1cJ4yQMcmxqbEVrDpqHd
</commit_message>
<xml_diff>
--- a/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
+++ b/sims/temporal_lp_economics_MODEL_v2_levered.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,10 @@
       <b val="1"/>
       <color rgb="00C53030"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C53030"/>
     </font>
   </fonts>
   <fills count="7">
@@ -134,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -177,6 +181,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -806,7 +811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -1025,6 +1030,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
@@ -1071,6 +1077,13 @@
       <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Rebuild pending operator go. Until then, read this sheet as a rough proxy, not the actual thing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>NB (entry 491): this faithfulness gap is ORTHOGONAL to the shape/steepness knob — the core issue is option PREMIUM income + a short-gamma (options) vol cost vs a spot proxy, regardless of m.</t>
         </is>
       </c>
     </row>

</xml_diff>